<commit_message>
feat(exports): update CSU 3-column header layout and centered footer date for student records exports
</commit_message>
<xml_diff>
--- a/tests/exports/empty_section_records.xlsx
+++ b/tests/exports/empty_section_records.xlsx
@@ -10,16 +10,27 @@
     <sheet name="Student Records" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Student Records'!$3:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Student Records'!$4:$5</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="8">
-  <si>
-    <t>CSU - Lal-lo Campus</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="10">
+  <si>
+    <t>REPUBLIC OF THE PHILIPPINES
+CAGAYAN STATE UNIVERSITY
+Andrews Campus, Tuguegarao City, Cagayan (Central Office)
+CSU Lal-lo Campus, Sta. Maria, Lal-lo, Cagayan (Sub Office)</t>
+  </si>
+  <si>
+    <t>Phone Number: 0945-0898-648
+Email Address: cicspadayaperformingartsguild@gmail.com
+Facebook page: CICS Padaya Performing Arts Guild</t>
+  </si>
+  <si>
+    <t>CAGAYAN STATE UNIVERSITY Lal-lo Campus</t>
   </si>
   <si>
     <t>#</t>
@@ -49,7 +60,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -60,11 +71,20 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="7.5"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <b val="1"/>
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
-      <sz val="14"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
@@ -104,12 +124,21 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -131,21 +160,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
@@ -155,6 +188,41 @@
   <dxfs count="0"/>
   <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="438150" cy="438150"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="CSU Logo" descr="CSU Logo"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="0"/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -448,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -458,63 +526,78 @@
     <col min="5" max="5" width="14" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" customHeight="1" ht="26">
+    <row r="1" spans="1:5" customHeight="1" ht="58">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" customHeight="1" ht="8"/>
-    <row r="3" spans="1:5" customHeight="1" ht="34">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="2" spans="1:5" customHeight="1" ht="24">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" spans="1:5" customHeight="1" ht="6"/>
+    <row r="4" spans="1:5" customHeight="1" ht="34">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="C4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>6</v>
       </c>
+      <c r="E4" s="4" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="4" spans="1:5" customHeight="1" ht="22">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" s="2"/>
+    <row r="5" spans="1:5" customHeight="1" ht="22">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="4"/>
     </row>
-    <row r="5" spans="1:5" customHeight="1" ht="24">
-      <c r="A5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="5"/>
+    <row r="6" spans="1:5" customHeight="1" ht="24">
+      <c r="A6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="6"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="7"/>
     </row>
   </sheetData>
   <mergeCells>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D3"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D4"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddFooter>&amp;LPrepared by: Admin Tester&amp;COctober 17, 2026&amp;RPage &amp;P of &amp;N</oddFooter>
-    <evenFooter>&amp;LPrepared by: Admin Tester&amp;COctober 17, 2026&amp;RPage &amp;P of &amp;N</evenFooter>
+    <oddFooter>&amp;LPrepared by: Admin Tester&amp;COctober 18, 2026&amp;R</oddFooter>
+    <evenFooter>&amp;LPrepared by: Admin Tester&amp;COctober 18, 2026&amp;R</evenFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(print): isolate modal printout in dedicated iframe to prevent duplicate pages and add 10 student seeders
</commit_message>
<xml_diff>
--- a/tests/exports/empty_section_records.xlsx
+++ b/tests/exports/empty_section_records.xlsx
@@ -25,9 +25,9 @@
 CSU Lal-lo Campus, Sta. Maria, Lal-lo, Cagayan (Sub Office)</t>
   </si>
   <si>
-    <t>Phone Number: 0945-0898-648
-Email Address: cicspadayaperformingartsguild@gmail.com
-Facebook page: CICS Padaya Performing Arts Guild</t>
+    <t>Phone Number:
+Email Address:
+Facebook page:</t>
   </si>
   <si>
     <t>CAGAYAN STATE UNIVERSITY Lal-lo Campus</t>
@@ -543,7 +543,7 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" customHeight="1" ht="6"/>
+    <row r="3" spans="1:5" customHeight="1" ht="12"/>
     <row r="4" spans="1:5" customHeight="1" ht="34">
       <c r="A4" s="4" t="s">
         <v>3</v>

</xml_diff>